<commit_message>
largest subarray and count of total subarrays with sum divisible by K
</commit_message>
<xml_diff>
--- a/DSA_sheet.xlsx
+++ b/DSA_sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PKIRANMU\Desktop\DSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ED9235B-B0D0-4E62-A7EB-53F415039F06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2068300-3E98-4789-AA97-44C6E27CDC86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,10 +24,10 @@
   </definedNames>
   <calcPr calcId="191028"/>
   <customWorkbookViews>
+    <customWorkbookView name="Filter 1" guid="{AAC291DF-A190-44CD-BE51-531E90BAF94B}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filter 3" guid="{1791E41F-2FB6-4B7D-BE94-80DC48681D60}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filter 2" guid="{64D3A7AF-0206-4BAD-A427-FE23D03476D4}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
     <customWorkbookView name="Filter 4" guid="{8391B649-8505-4799-A195-AB43CB26E425}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filter 2" guid="{64D3A7AF-0206-4BAD-A427-FE23D03476D4}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filter 3" guid="{1791E41F-2FB6-4B7D-BE94-80DC48681D60}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filter 1" guid="{AAC291DF-A190-44CD-BE51-531E90BAF94B}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1259" uniqueCount="701">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1261" uniqueCount="701">
   <si>
     <t>DSA by Shradha Ma'am</t>
   </si>
@@ -3848,7 +3848,9 @@
         <v>57</v>
       </c>
       <c r="C30" s="11"/>
-      <c r="D30" s="41"/>
+      <c r="D30" s="40" t="s">
+        <v>700</v>
+      </c>
       <c r="E30" s="12" t="s">
         <v>58</v>
       </c>
@@ -3885,7 +3887,9 @@
         <v>59</v>
       </c>
       <c r="C31" s="11"/>
-      <c r="D31" s="41"/>
+      <c r="D31" s="40" t="s">
+        <v>700</v>
+      </c>
       <c r="E31" s="12" t="s">
         <v>53</v>
       </c>
@@ -33221,21 +33225,21 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{AAC291DF-A190-44CD-BE51-531E90BAF94B}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{64D3A7AF-0206-4BAD-A427-FE23D03476D4}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A293:C332" xr:uid="{898F705B-02E1-4035-9DAF-28A2957768D4}"/>
+      <autoFilter ref="A11:C37" xr:uid="{6C22C7A1-77C1-4B2F-A1BF-1C69FA90CF8D}"/>
+    </customSheetView>
+    <customSheetView guid="{1791E41F-2FB6-4B7D-BE94-80DC48681D60}" filter="1" showAutoFilter="1">
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+      <autoFilter ref="A11:D37" xr:uid="{F2FC3DB7-F7D9-4483-A689-303110D9EEF7}"/>
     </customSheetView>
     <customSheetView guid="{8391B649-8505-4799-A195-AB43CB26E425}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A11:D37" xr:uid="{20DB233E-3794-4A76-8E31-12DBB885B708}"/>
+      <autoFilter ref="A11:D37" xr:uid="{5BF779D7-6B26-455E-8906-8CA3FA91EB8C}"/>
     </customSheetView>
-    <customSheetView guid="{1791E41F-2FB6-4B7D-BE94-80DC48681D60}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{AAC291DF-A190-44CD-BE51-531E90BAF94B}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A11:D37" xr:uid="{854A1D4E-9F62-4B90-AE3B-02D1CCDB816A}"/>
-    </customSheetView>
-    <customSheetView guid="{64D3A7AF-0206-4BAD-A427-FE23D03476D4}" filter="1" showAutoFilter="1">
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A11:C37" xr:uid="{81478CA2-2CCA-4B0B-B3F6-3C259D7E355A}"/>
+      <autoFilter ref="A293:C332" xr:uid="{F6F1C060-78DE-470C-9F69-7870C67EECC1}"/>
     </customSheetView>
   </customSheetViews>
   <mergeCells count="1">

</xml_diff>

<commit_message>
String DSA Initial Commit
</commit_message>
<xml_diff>
--- a/DSA_sheet.xlsx
+++ b/DSA_sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PKIRANMU\Desktop\DSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2068300-3E98-4789-AA97-44C6E27CDC86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9289EA70-EA1E-4FD1-A2AB-4E83A7211DB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,10 +24,10 @@
   </definedNames>
   <calcPr calcId="191028"/>
   <customWorkbookViews>
+    <customWorkbookView name="Filter 4" guid="{8391B649-8505-4799-A195-AB43CB26E425}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filter 2" guid="{64D3A7AF-0206-4BAD-A427-FE23D03476D4}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filter 3" guid="{1791E41F-2FB6-4B7D-BE94-80DC48681D60}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
     <customWorkbookView name="Filter 1" guid="{AAC291DF-A190-44CD-BE51-531E90BAF94B}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filter 3" guid="{1791E41F-2FB6-4B7D-BE94-80DC48681D60}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filter 2" guid="{64D3A7AF-0206-4BAD-A427-FE23D03476D4}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filter 4" guid="{8391B649-8505-4799-A195-AB43CB26E425}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1261" uniqueCount="701">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1266" uniqueCount="701">
   <si>
     <t>DSA by Shradha Ma'am</t>
   </si>
@@ -3926,7 +3926,9 @@
         <v>60</v>
       </c>
       <c r="C32" s="11"/>
-      <c r="D32" s="41"/>
+      <c r="D32" s="40" t="s">
+        <v>700</v>
+      </c>
       <c r="E32" s="12" t="s">
         <v>61</v>
       </c>
@@ -4025,7 +4027,9 @@
         <v>63</v>
       </c>
       <c r="C35" s="11"/>
-      <c r="D35" s="41"/>
+      <c r="D35" s="40" t="s">
+        <v>700</v>
+      </c>
       <c r="E35" s="12" t="s">
         <v>64</v>
       </c>
@@ -4062,7 +4066,9 @@
         <v>65</v>
       </c>
       <c r="C36" s="11"/>
-      <c r="D36" s="41"/>
+      <c r="D36" s="40" t="s">
+        <v>700</v>
+      </c>
       <c r="E36" s="12" t="s">
         <v>66</v>
       </c>
@@ -4099,7 +4105,9 @@
         <v>67</v>
       </c>
       <c r="C37" s="11"/>
-      <c r="D37" s="41"/>
+      <c r="D37" s="40" t="s">
+        <v>700</v>
+      </c>
       <c r="E37" s="12" t="s">
         <v>51</v>
       </c>
@@ -4138,7 +4146,9 @@
         <v>69</v>
       </c>
       <c r="C38" s="11"/>
-      <c r="D38" s="41"/>
+      <c r="D38" s="40" t="s">
+        <v>700</v>
+      </c>
       <c r="E38" s="12" t="s">
         <v>70</v>
       </c>
@@ -33225,21 +33235,21 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{64D3A7AF-0206-4BAD-A427-FE23D03476D4}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{AAC291DF-A190-44CD-BE51-531E90BAF94B}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A11:C37" xr:uid="{6C22C7A1-77C1-4B2F-A1BF-1C69FA90CF8D}"/>
+      <autoFilter ref="A293:C332" xr:uid="{1D98FFF6-E0E2-458A-A419-745DCE61C4A3}"/>
+    </customSheetView>
+    <customSheetView guid="{8391B649-8505-4799-A195-AB43CB26E425}" filter="1" showAutoFilter="1">
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+      <autoFilter ref="A11:D37" xr:uid="{D9D9B8AB-A8C8-45EA-B11F-318B0A501882}"/>
     </customSheetView>
     <customSheetView guid="{1791E41F-2FB6-4B7D-BE94-80DC48681D60}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A11:D37" xr:uid="{F2FC3DB7-F7D9-4483-A689-303110D9EEF7}"/>
+      <autoFilter ref="A11:D37" xr:uid="{3C337885-E174-4DBD-9621-A0309ACB5DA4}"/>
     </customSheetView>
-    <customSheetView guid="{8391B649-8505-4799-A195-AB43CB26E425}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{64D3A7AF-0206-4BAD-A427-FE23D03476D4}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A11:D37" xr:uid="{5BF779D7-6B26-455E-8906-8CA3FA91EB8C}"/>
-    </customSheetView>
-    <customSheetView guid="{AAC291DF-A190-44CD-BE51-531E90BAF94B}" filter="1" showAutoFilter="1">
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A293:C332" xr:uid="{F6F1C060-78DE-470C-9F69-7870C67EECC1}"/>
+      <autoFilter ref="A11:C37" xr:uid="{DE171A5D-6230-4F52-BEDD-19F79CEA467C}"/>
     </customSheetView>
   </customSheetViews>
   <mergeCells count="1">

</xml_diff>